<commit_message>
llm 3 versiooni ja thread_level päring
</commit_message>
<xml_diff>
--- a/data/gold_standard_filled.xlsx
+++ b/data/gold_standard_filled.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\annmarle\Desktop\Redditi postituste automaatne klassifitseerimine erineva signaalitasemega keskkondades\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{05D7641C-AA21-4FE7-8020-A005326A2E90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29B98BE6-F925-4321-8965-DD91BD8F3AA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="14040" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1831,12 +1831,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2147,7 +2146,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2168,7 +2167,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2179,7 +2178,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="144" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -2201,7 +2200,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2231,7 +2230,7 @@
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
@@ -2267,7 +2266,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -2553,7 +2552,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>75</v>
       </c>
@@ -2619,7 +2618,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>87</v>
       </c>
@@ -2696,7 +2695,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>101</v>
       </c>
@@ -2982,7 +2981,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>153</v>
       </c>
@@ -3125,7 +3124,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>178</v>
       </c>
@@ -3136,7 +3135,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>180</v>
       </c>
@@ -3180,7 +3179,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>187</v>
       </c>
@@ -3191,7 +3190,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>189</v>
       </c>
@@ -3232,7 +3231,7 @@
         <v>196</v>
       </c>
       <c r="C99" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="144" x14ac:dyDescent="0.3">
@@ -3301,7 +3300,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="106" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:3" ht="144" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>209</v>
       </c>
@@ -3389,7 +3388,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="114" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:3" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>225</v>
       </c>
@@ -3422,7 +3421,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="117" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>231</v>
       </c>
@@ -3433,7 +3432,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="118" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>233</v>
       </c>
@@ -3444,7 +3443,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="119" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>235</v>
       </c>
@@ -3466,7 +3465,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="121" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>239</v>
       </c>
@@ -3477,7 +3476,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>241</v>
       </c>
@@ -3488,7 +3487,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="123" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>243</v>
       </c>
@@ -3540,7 +3539,7 @@
         <v>252</v>
       </c>
       <c r="C127" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="128" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -3554,7 +3553,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="129" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>255</v>
       </c>
@@ -3598,7 +3597,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="133" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>263</v>
       </c>
@@ -3617,7 +3616,7 @@
         <v>266</v>
       </c>
       <c r="C134" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="135" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
@@ -3631,7 +3630,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>269</v>
       </c>
@@ -3642,7 +3641,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="137" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>271</v>
       </c>
@@ -3653,7 +3652,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>273</v>
       </c>
@@ -3686,7 +3685,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>279</v>
       </c>
@@ -3705,7 +3704,7 @@
         <v>282</v>
       </c>
       <c r="C142" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="143" spans="1:3" ht="144" x14ac:dyDescent="0.3">
@@ -3730,7 +3729,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="145" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>287</v>
       </c>
@@ -3752,7 +3751,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>291</v>
       </c>
@@ -3763,7 +3762,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="148" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>293</v>
       </c>
@@ -3785,7 +3784,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>297</v>
       </c>
@@ -3796,7 +3795,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="151" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>299</v>
       </c>
@@ -3851,7 +3850,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>309</v>
       </c>
@@ -3862,7 +3861,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>311</v>
       </c>
@@ -3884,7 +3883,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>315</v>
       </c>
@@ -3895,7 +3894,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="160" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>317</v>
       </c>
@@ -3906,7 +3905,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>319</v>
       </c>
@@ -3917,7 +3916,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>321</v>
       </c>
@@ -3928,7 +3927,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="163" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>323</v>
       </c>
@@ -3950,7 +3949,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="165" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>327</v>
       </c>
@@ -3972,7 +3971,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>331</v>
       </c>
@@ -3994,7 +3993,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="169" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>334</v>
       </c>
@@ -4038,7 +4037,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>342</v>
       </c>
@@ -4060,7 +4059,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>346</v>
       </c>
@@ -4071,7 +4070,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="176" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>347</v>
       </c>
@@ -4115,7 +4114,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="180" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>355</v>
       </c>
@@ -4137,7 +4136,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>359</v>
       </c>
@@ -4148,7 +4147,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="183" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>361</v>
       </c>
@@ -4159,7 +4158,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="184" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>363</v>
       </c>
@@ -4192,7 +4191,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="187" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>369</v>
       </c>
@@ -4247,7 +4246,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>379</v>
       </c>
@@ -4280,7 +4279,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="195" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>385</v>
       </c>
@@ -4291,7 +4290,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="196" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>387</v>
       </c>
@@ -4302,7 +4301,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="197" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:3" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>389</v>
       </c>
@@ -4423,7 +4422,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="208" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>411</v>
       </c>
@@ -4434,7 +4433,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>413</v>
       </c>
@@ -4445,7 +4444,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="210" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>415</v>
       </c>
@@ -4456,7 +4455,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="211" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>417</v>
       </c>
@@ -4475,7 +4474,7 @@
         <v>420</v>
       </c>
       <c r="C212" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="213" spans="1:3" ht="72" x14ac:dyDescent="0.3">
@@ -4511,7 +4510,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>427</v>
       </c>
@@ -4533,7 +4532,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>431</v>
       </c>
@@ -4544,7 +4543,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="219" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>433</v>
       </c>
@@ -4555,7 +4554,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="220" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:3" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>435</v>
       </c>
@@ -4566,7 +4565,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="221" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>437</v>
       </c>
@@ -4621,7 +4620,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="226" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>447</v>
       </c>
@@ -4632,7 +4631,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="227" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>449</v>
       </c>
@@ -4654,7 +4653,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="229" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>453</v>
       </c>
@@ -4665,7 +4664,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>455</v>
       </c>
@@ -4698,7 +4697,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>461</v>
       </c>
@@ -4709,7 +4708,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="234" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>463</v>
       </c>
@@ -4753,7 +4752,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="238" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:3" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>471</v>
       </c>
@@ -4808,7 +4807,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="243" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>481</v>
       </c>
@@ -4995,7 +4994,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="260" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>515</v>
       </c>
@@ -5006,7 +5005,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="261" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>517</v>
       </c>
@@ -5039,7 +5038,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="264" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>523</v>
       </c>
@@ -5050,7 +5049,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="265" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:3" ht="144" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>525</v>
       </c>
@@ -5072,7 +5071,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="267" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>529</v>
       </c>
@@ -5116,7 +5115,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="271" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>537</v>
       </c>
@@ -5138,7 +5137,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="273" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>541</v>
       </c>
@@ -5193,7 +5192,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="278" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>551</v>
       </c>
@@ -5204,7 +5203,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="279" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>553</v>
       </c>
@@ -5281,7 +5280,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="286" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>567</v>
       </c>
@@ -5292,7 +5291,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="287" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>569</v>
       </c>
@@ -5303,7 +5302,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="288" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>571</v>
       </c>
@@ -5336,7 +5335,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="291" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>577</v>
       </c>
@@ -5399,7 +5398,7 @@
         <v>588</v>
       </c>
       <c r="C296" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
   </sheetData>

</xml_diff>